<commit_message>
Simplify Kennedy November: full night-float week 11/1-6, drop Friday handoff
Per PD: give Kennedy the whole first November week on night float (11/1-6)
+ off the 11/7-8 weekend, and let the PD arrange the Friday-11/6 travel swap
by hand. Drops the Chiasson/Mullins Friday handoff, removing 5 exceptions
(down to 7 accepted accommodation costs, mostly on non-LSH interns).
Oghenesume keeps his 4/10-11 weekend off; PD can hand-switch his 4/9/4/12
short calls if more is wanted. Regenerated year artifacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>MULLINS</t>
+          <t>CHIASSON</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>WISE, KENNEDY</t>
+          <t>WISE, MULLINS</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert Kennedy<->Chiasson November swap per PD (back to pure march)
Disabled KEN_SWAP_DAYS. November returns to the deterministic march: Chiasson
holds the 11/1-6 night float, Kennedy on his normal schedule (own NF week
11/8-13). Thanksgiving 11/26 still off. Base audit back to 5 documented
exceptions; other approved accommodations (Bronson Christmas, Oghenesume
Jan/Apr, MacNeille Oct) unchanged. Regenerated year artifacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
@@ -3113,7 +3113,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, MULLINS</t>
+          <t>KENNEDY, MULLINS</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3153,17 +3153,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3183,12 +3183,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>WISE, CHIASSON</t>
+          <t>WISE, KENNEDY</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3208,12 +3208,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U, WISE</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U, WISE</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3325,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, WISE</t>
+          <t>CHIASSON, WISE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3350,12 +3350,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, SAEED U</t>
+          <t>CHIASSON, SAEED U</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3370,17 +3370,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3400,12 +3400,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, WISE</t>
+          <t>CHIASSON, WISE</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kennedy: night float the first week of November (11/1-6)
Re-enabled KEN_SWAP_DAYS so Kennedy holds NF Sun 11/1 - Fri 11/6, off the
11/7-8 weekend. Chiasson takes his 11/8-13 night-float week in return (she
holds the 11/1-6 nights, so the trade is unavoidable). Thanksgiving 11/26
off. Regenerated year artifacts.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01J6EM8SxuZs5C898HeFBgt7
</commit_message>
<xml_diff>
--- a/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
+++ b/intern_schedule_2026-2027/schedules/TYP_Intern_Schedule_Sep2026-Jun2027.xlsx
@@ -3113,7 +3113,7 @@
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3133,12 +3133,12 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY, MULLINS</t>
+          <t>CHIASSON, MULLINS</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3153,17 +3153,17 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3183,12 +3183,12 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>WISE, KENNEDY</t>
+          <t>WISE, CHIASSON</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON</t>
+          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3208,12 +3208,12 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3228,17 +3228,17 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
+          <t>CHIASSON</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>WISE, MULLINS</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
           <t>KENNEDY</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>WISE, MULLINS</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3295,17 +3295,17 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U, WISE</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U, WISE</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3325,12 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, WISE</t>
+          <t>KENNEDY, WISE</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3350,12 +3350,12 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, SAEED U</t>
+          <t>KENNEDY, SAEED U</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>
@@ -3370,17 +3370,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
+          <t>KENNEDY</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>SAEED U</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>CHIASSON</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>SAEED U</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>KENNEDY</t>
         </is>
       </c>
     </row>
@@ -3400,12 +3400,12 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>CHIASSON, WISE</t>
+          <t>KENNEDY, WISE</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>KENNEDY</t>
+          <t>CHIASSON</t>
         </is>
       </c>
     </row>

</xml_diff>